<commit_message>
excel file date format
</commit_message>
<xml_diff>
--- a/public/download/product_format.xlsx
+++ b/public/download/product_format.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="itemExcelImport" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -270,7 +270,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1048576"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultColWidth="9.171875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.72"/>
@@ -281,7 +281,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.98"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -313,12 +313,15 @@
       <c r="F2" s="5"/>
       <c r="G2" s="6"/>
     </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G1:G1001" type="none">
-      <formula1>12/30/1899</formula1>
-      <formula2>12/30/1899</formula2>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F1:F1001" type="list">
+      <formula1>"Stand Only,Online Only,Stand And Online"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G1:G1001" type="date">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>